<commit_message>
USB cable and adapter added in BOM
</commit_message>
<xml_diff>
--- a/Photo_frame_v_1.0/Deliverables/BOM/Client_BOM.xlsx
+++ b/Photo_frame_v_1.0/Deliverables/BOM/Client_BOM.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="219">
   <si>
     <t>#</t>
   </si>
@@ -678,6 +678,12 @@
   </si>
   <si>
     <t xml:space="preserve"> IPS ILI9488 No Touch</t>
+  </si>
+  <si>
+    <t>USB cable and Adapter</t>
+  </si>
+  <si>
+    <t>Charging cable and Adapter for 100watt USB PD support</t>
   </si>
 </sst>
 </file>
@@ -1786,7 +1792,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.14285714285714" style="1" customWidth="1"/>
@@ -1879,7 +1885,7 @@
       </c>
       <c r="K3" s="9"/>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" ht="15.75" spans="1:11">
       <c r="A4" s="2"/>
       <c r="B4" s="7">
         <f>ROW(B4)-ROW($B$2)</f>
@@ -2451,7 +2457,7 @@
       </c>
       <c r="K21" s="9"/>
     </row>
-    <row r="22" spans="1:11">
+    <row r="22" ht="15.75" spans="1:11">
       <c r="A22" s="2"/>
       <c r="B22" s="7">
         <f>ROW(B22)-ROW($B$2)</f>
@@ -2483,7 +2489,7 @@
       </c>
       <c r="K22" s="11"/>
     </row>
-    <row r="23" spans="1:11">
+    <row r="23" ht="15.75" spans="1:11">
       <c r="A23" s="2"/>
       <c r="B23" s="7">
         <f>ROW(B23)-ROW($B$2)</f>
@@ -2515,7 +2521,7 @@
       </c>
       <c r="K23" s="9"/>
     </row>
-    <row r="24" spans="1:11">
+    <row r="24" ht="15.75" spans="1:11">
       <c r="A24" s="2"/>
       <c r="B24" s="7">
         <f>ROW(B24)-ROW($B$2)</f>
@@ -2579,7 +2585,7 @@
       </c>
       <c r="K25" s="9"/>
     </row>
-    <row r="26" spans="1:11">
+    <row r="26" ht="15.75" spans="1:11">
       <c r="A26" s="2"/>
       <c r="B26" s="7">
         <f>ROW(B26)-ROW($B$2)</f>
@@ -2835,7 +2841,7 @@
       </c>
       <c r="K33" s="9"/>
     </row>
-    <row r="34" spans="1:11">
+    <row r="34" ht="15.75" spans="1:11">
       <c r="A34" s="2"/>
       <c r="B34" s="7">
         <f>ROW(B34)-ROW($B$2)</f>
@@ -2867,7 +2873,7 @@
       </c>
       <c r="K34" s="11"/>
     </row>
-    <row r="35" spans="1:11">
+    <row r="35" ht="15.75" spans="1:11">
       <c r="A35" s="2"/>
       <c r="B35" s="7">
         <f>ROW(B35)-ROW($B$2)</f>
@@ -2963,7 +2969,7 @@
       </c>
       <c r="K37" s="9"/>
     </row>
-    <row r="38" spans="1:11">
+    <row r="38" ht="15.75" spans="1:11">
       <c r="A38" s="2"/>
       <c r="B38" s="7">
         <f>ROW(B38)-ROW($B$2)</f>
@@ -2995,7 +3001,7 @@
       </c>
       <c r="K38" s="11"/>
     </row>
-    <row r="39" spans="1:11">
+    <row r="39" ht="15.75" spans="1:11">
       <c r="A39" s="2"/>
       <c r="B39" s="7">
         <f>ROW(B39)-ROW($B$2)</f>
@@ -3122,6 +3128,38 @@
         <v>1</v>
       </c>
       <c r="K42" s="9"/>
+    </row>
+    <row r="43" ht="24.75" spans="1:11">
+      <c r="A43" s="2"/>
+      <c r="B43" s="7">
+        <f>ROW(B43)-ROW($B$2)</f>
+        <v>41</v>
+      </c>
+      <c r="C43" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="E43" s="10" t="s">
+        <v>218</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="G43" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="H43" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="I43" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="J43" s="9">
+        <v>1</v>
+      </c>
+      <c r="K43" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
#7 Peripherals link added in Client BOM.
</commit_message>
<xml_diff>
--- a/Photo_frame_v_1.0/Deliverables/BOM/Client_BOM.xlsx
+++ b/Photo_frame_v_1.0/Deliverables/BOM/Client_BOM.xlsx
@@ -1,15 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\umarkhan-photoframe\Photo_frame_v_1.0\Deliverables\BOM\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="19635" windowHeight="7620"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19635" windowHeight="7620"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -27,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="221">
   <si>
     <t>#</t>
   </si>
@@ -684,19 +689,19 @@
   </si>
   <si>
     <t>Charging cable and Adapter for 100watt USB PD support</t>
+  </si>
+  <si>
+    <t>Aliexpress Note: Selection from link options: IPS ILI9488 No Touch</t>
+  </si>
+  <si>
+    <t>Taobao (Note: 100W Charger Select Type 2C1A</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="25">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -744,147 +749,10 @@
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -903,194 +771,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="16">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -1181,253 +863,14 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1467,68 +910,28 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="0003A4CB"/>
-      <color rgb="002CD0B2"/>
+      <color rgb="FF03A4CB"/>
+      <color rgb="FF2CD0B2"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1786,28 +1189,29 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:K43"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="3.14285714285714" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.7142857142857" style="1" customWidth="1"/>
+    <col min="2" max="2" width="3.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="36" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5714285714286" customWidth="1"/>
-    <col min="7" max="7" width="33.4285714285714" customWidth="1"/>
-    <col min="8" max="8" width="21.4285714285714" customWidth="1"/>
-    <col min="9" max="9" width="17.8571428571429" customWidth="1"/>
-    <col min="10" max="10" width="16.7142857142857" customWidth="1"/>
-    <col min="11" max="11" width="29.4285714285714" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" customWidth="1"/>
+    <col min="9" max="9" width="17.85546875" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" customWidth="1"/>
+    <col min="11" max="11" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" spans="1:11">
+    <row r="1" spans="1:11">
       <c r="A1" s="2"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1820,7 +1224,7 @@
       <c r="J1" s="14"/>
       <c r="K1" s="14"/>
     </row>
-    <row r="2" ht="15.75" spans="1:11">
+    <row r="2" spans="1:11">
       <c r="A2" s="2"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1853,10 +1257,10 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" ht="24.75" spans="1:11">
+    <row r="3" spans="1:11" ht="24">
       <c r="A3" s="2"/>
       <c r="B3" s="7">
-        <f>ROW(B3)-ROW($B$2)</f>
+        <f t="shared" ref="B3:B43" si="0">ROW(B3)-ROW($B$2)</f>
         <v>1</v>
       </c>
       <c r="C3" s="8" t="s">
@@ -1885,10 +1289,10 @@
       </c>
       <c r="K3" s="9"/>
     </row>
-    <row r="4" ht="15.75" spans="1:11">
+    <row r="4" spans="1:11">
       <c r="A4" s="2"/>
       <c r="B4" s="7">
-        <f>ROW(B4)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="C4" s="8" t="s">
@@ -1917,10 +1321,10 @@
       </c>
       <c r="K4" s="11"/>
     </row>
-    <row r="5" ht="36.75" spans="1:11">
+    <row r="5" spans="1:11" ht="36">
       <c r="A5" s="2"/>
       <c r="B5" s="7">
-        <f>ROW(B5)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C5" s="13" t="s">
@@ -1949,10 +1353,10 @@
       </c>
       <c r="K5" s="9"/>
     </row>
-    <row r="6" ht="15.75" spans="1:11">
+    <row r="6" spans="1:11">
       <c r="A6" s="2"/>
       <c r="B6" s="7">
-        <f>ROW(B6)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C6" s="8"/>
@@ -1979,10 +1383,10 @@
       </c>
       <c r="K6" s="11"/>
     </row>
-    <row r="7" ht="15.75" spans="1:11">
+    <row r="7" spans="1:11">
       <c r="A7" s="2"/>
       <c r="B7" s="7">
-        <f>ROW(B7)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C7" s="13" t="s">
@@ -2011,10 +1415,10 @@
       </c>
       <c r="K7" s="9"/>
     </row>
-    <row r="8" ht="24.75" spans="1:11">
+    <row r="8" spans="1:11" ht="24">
       <c r="A8" s="2"/>
       <c r="B8" s="7">
-        <f>ROW(B8)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C8" s="8" t="s">
@@ -2043,10 +1447,10 @@
       </c>
       <c r="K8" s="11"/>
     </row>
-    <row r="9" ht="15.75" spans="1:11">
+    <row r="9" spans="1:11">
       <c r="A9" s="2"/>
       <c r="B9" s="7">
-        <f>ROW(B9)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C9" s="13" t="s">
@@ -2075,10 +1479,10 @@
       </c>
       <c r="K9" s="9"/>
     </row>
-    <row r="10" ht="15.75" spans="1:11">
+    <row r="10" spans="1:11">
       <c r="A10" s="2"/>
       <c r="B10" s="7">
-        <f>ROW(B10)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C10" s="8" t="s">
@@ -2107,10 +1511,10 @@
       </c>
       <c r="K10" s="11"/>
     </row>
-    <row r="11" ht="15.75" spans="1:11">
+    <row r="11" spans="1:11">
       <c r="A11" s="2"/>
       <c r="B11" s="7">
-        <f>ROW(B11)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C11" s="13"/>
@@ -2137,10 +1541,10 @@
       </c>
       <c r="K11" s="9"/>
     </row>
-    <row r="12" ht="24.75" spans="1:11">
+    <row r="12" spans="1:11" ht="24">
       <c r="A12" s="2"/>
       <c r="B12" s="7">
-        <f>ROW(B12)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C12" s="8" t="s">
@@ -2169,10 +1573,10 @@
       </c>
       <c r="K12" s="11"/>
     </row>
-    <row r="13" ht="24.75" spans="1:11">
+    <row r="13" spans="1:11" ht="36">
       <c r="A13" s="2"/>
       <c r="B13" s="7">
-        <f>ROW(B13)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C13" s="13" t="s">
@@ -2201,10 +1605,10 @@
       </c>
       <c r="K13" s="9"/>
     </row>
-    <row r="14" ht="24.75" spans="1:11">
+    <row r="14" spans="1:11" ht="24">
       <c r="A14" s="2"/>
       <c r="B14" s="7">
-        <f>ROW(B14)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C14" s="8" t="s">
@@ -2233,10 +1637,10 @@
       </c>
       <c r="K14" s="11"/>
     </row>
-    <row r="15" ht="72.75" spans="1:11">
+    <row r="15" spans="1:11" ht="72">
       <c r="A15" s="2"/>
       <c r="B15" s="7">
-        <f>ROW(B15)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C15" s="13" t="s">
@@ -2265,10 +1669,10 @@
       </c>
       <c r="K15" s="9"/>
     </row>
-    <row r="16" ht="24.75" spans="1:11">
+    <row r="16" spans="1:11" ht="36">
       <c r="A16" s="2"/>
       <c r="B16" s="7">
-        <f>ROW(B16)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C16" s="8" t="s">
@@ -2297,10 +1701,10 @@
       </c>
       <c r="K16" s="11"/>
     </row>
-    <row r="17" ht="24.75" spans="1:11">
+    <row r="17" spans="1:11" ht="24">
       <c r="A17" s="2"/>
       <c r="B17" s="7">
-        <f>ROW(B17)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="C17" s="13" t="s">
@@ -2329,10 +1733,10 @@
       </c>
       <c r="K17" s="9"/>
     </row>
-    <row r="18" ht="24.75" spans="1:11">
+    <row r="18" spans="1:11" ht="24">
       <c r="A18" s="2"/>
       <c r="B18" s="7">
-        <f>ROW(B18)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C18" s="8" t="s">
@@ -2361,10 +1765,10 @@
       </c>
       <c r="K18" s="11"/>
     </row>
-    <row r="19" ht="409.5" spans="1:11">
+    <row r="19" spans="1:11" ht="409.5">
       <c r="A19" s="2"/>
       <c r="B19" s="7">
-        <f>ROW(B19)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C19" s="13" t="s">
@@ -2393,10 +1797,10 @@
       </c>
       <c r="K19" s="9"/>
     </row>
-    <row r="20" ht="24.75" spans="1:11">
+    <row r="20" spans="1:11" ht="24">
       <c r="A20" s="2"/>
       <c r="B20" s="7">
-        <f>ROW(B20)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C20" s="8" t="s">
@@ -2425,10 +1829,10 @@
       </c>
       <c r="K20" s="11"/>
     </row>
-    <row r="21" ht="24.75" spans="1:11">
+    <row r="21" spans="1:11" ht="24">
       <c r="A21" s="2"/>
       <c r="B21" s="7">
-        <f>ROW(B21)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="C21" s="13" t="s">
@@ -2457,10 +1861,10 @@
       </c>
       <c r="K21" s="9"/>
     </row>
-    <row r="22" ht="15.75" spans="1:11">
+    <row r="22" spans="1:11">
       <c r="A22" s="2"/>
       <c r="B22" s="7">
-        <f>ROW(B22)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C22" s="8" t="s">
@@ -2489,10 +1893,10 @@
       </c>
       <c r="K22" s="11"/>
     </row>
-    <row r="23" ht="15.75" spans="1:11">
+    <row r="23" spans="1:11">
       <c r="A23" s="2"/>
       <c r="B23" s="7">
-        <f>ROW(B23)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="C23" s="13" t="s">
@@ -2521,10 +1925,10 @@
       </c>
       <c r="K23" s="9"/>
     </row>
-    <row r="24" ht="15.75" spans="1:11">
+    <row r="24" spans="1:11">
       <c r="A24" s="2"/>
       <c r="B24" s="7">
-        <f>ROW(B24)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="C24" s="8" t="s">
@@ -2553,10 +1957,10 @@
       </c>
       <c r="K24" s="11"/>
     </row>
-    <row r="25" ht="24.75" spans="1:11">
+    <row r="25" spans="1:11" ht="24">
       <c r="A25" s="2"/>
       <c r="B25" s="7">
-        <f>ROW(B25)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="C25" s="8" t="s">
@@ -2585,10 +1989,10 @@
       </c>
       <c r="K25" s="9"/>
     </row>
-    <row r="26" ht="15.75" spans="1:11">
+    <row r="26" spans="1:11">
       <c r="A26" s="2"/>
       <c r="B26" s="7">
-        <f>ROW(B26)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C26" s="8" t="s">
@@ -2617,10 +2021,10 @@
       </c>
       <c r="K26" s="11"/>
     </row>
-    <row r="27" ht="15.75" spans="1:11">
+    <row r="27" spans="1:11">
       <c r="A27" s="2"/>
       <c r="B27" s="7">
-        <f>ROW(B27)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="C27" s="13" t="s">
@@ -2649,10 +2053,10 @@
       </c>
       <c r="K27" s="9"/>
     </row>
-    <row r="28" ht="15.75" spans="1:11">
+    <row r="28" spans="1:11">
       <c r="A28" s="2"/>
       <c r="B28" s="7">
-        <f>ROW(B28)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="C28" s="8" t="s">
@@ -2681,10 +2085,10 @@
       </c>
       <c r="K28" s="11"/>
     </row>
-    <row r="29" ht="15.75" spans="1:11">
+    <row r="29" spans="1:11">
       <c r="A29" s="2"/>
       <c r="B29" s="7">
-        <f>ROW(B29)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="C29" s="13" t="s">
@@ -2713,10 +2117,10 @@
       </c>
       <c r="K29" s="9"/>
     </row>
-    <row r="30" ht="24.75" spans="1:11">
+    <row r="30" spans="1:11" ht="24">
       <c r="A30" s="2"/>
       <c r="B30" s="7">
-        <f>ROW(B30)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C30" s="8" t="s">
@@ -2745,10 +2149,10 @@
       </c>
       <c r="K30" s="11"/>
     </row>
-    <row r="31" ht="15.75" spans="1:11">
+    <row r="31" spans="1:11">
       <c r="A31" s="2"/>
       <c r="B31" s="7">
-        <f>ROW(B31)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>29</v>
       </c>
       <c r="C31" s="13" t="s">
@@ -2777,10 +2181,10 @@
       </c>
       <c r="K31" s="9"/>
     </row>
-    <row r="32" ht="15.75" spans="1:11">
+    <row r="32" spans="1:11">
       <c r="A32" s="2"/>
       <c r="B32" s="7">
-        <f>ROW(B32)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C32" s="8" t="s">
@@ -2809,10 +2213,10 @@
       </c>
       <c r="K32" s="11"/>
     </row>
-    <row r="33" ht="36.75" spans="1:11">
+    <row r="33" spans="1:11" ht="36">
       <c r="A33" s="2"/>
       <c r="B33" s="7">
-        <f>ROW(B33)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="C33" s="13" t="s">
@@ -2841,10 +2245,10 @@
       </c>
       <c r="K33" s="9"/>
     </row>
-    <row r="34" ht="15.75" spans="1:11">
+    <row r="34" spans="1:11">
       <c r="A34" s="2"/>
       <c r="B34" s="7">
-        <f>ROW(B34)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C34" s="8" t="s">
@@ -2873,10 +2277,10 @@
       </c>
       <c r="K34" s="11"/>
     </row>
-    <row r="35" ht="15.75" spans="1:11">
+    <row r="35" spans="1:11">
       <c r="A35" s="2"/>
       <c r="B35" s="7">
-        <f>ROW(B35)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="C35" s="13" t="s">
@@ -2905,10 +2309,10 @@
       </c>
       <c r="K35" s="9"/>
     </row>
-    <row r="36" ht="36.75" spans="1:11">
+    <row r="36" spans="1:11" ht="36">
       <c r="A36" s="2"/>
       <c r="B36" s="7">
-        <f>ROW(B36)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>34</v>
       </c>
       <c r="C36" s="8" t="s">
@@ -2937,10 +2341,10 @@
       </c>
       <c r="K36" s="11"/>
     </row>
-    <row r="37" ht="24.75" spans="1:11">
+    <row r="37" spans="1:11" ht="24">
       <c r="A37" s="2"/>
       <c r="B37" s="7">
-        <f>ROW(B37)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>35</v>
       </c>
       <c r="C37" s="8" t="s">
@@ -2969,10 +2373,10 @@
       </c>
       <c r="K37" s="9"/>
     </row>
-    <row r="38" ht="15.75" spans="1:11">
+    <row r="38" spans="1:11">
       <c r="A38" s="2"/>
       <c r="B38" s="7">
-        <f>ROW(B38)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>36</v>
       </c>
       <c r="C38" s="8" t="s">
@@ -3001,10 +2405,10 @@
       </c>
       <c r="K38" s="11"/>
     </row>
-    <row r="39" ht="15.75" spans="1:11">
+    <row r="39" spans="1:11">
       <c r="A39" s="2"/>
       <c r="B39" s="7">
-        <f>ROW(B39)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>37</v>
       </c>
       <c r="C39" s="13" t="s">
@@ -3033,10 +2437,10 @@
       </c>
       <c r="K39" s="9"/>
     </row>
-    <row r="40" ht="24.75" spans="1:11">
+    <row r="40" spans="1:11" ht="36">
       <c r="A40" s="2"/>
       <c r="B40" s="7">
-        <f>ROW(B40)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>38</v>
       </c>
       <c r="C40" s="8" t="s">
@@ -3065,10 +2469,10 @@
       </c>
       <c r="K40" s="11"/>
     </row>
-    <row r="41" ht="15.75" spans="1:11">
+    <row r="41" spans="1:11">
       <c r="A41" s="2"/>
       <c r="B41" s="7">
-        <f>ROW(B41)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>39</v>
       </c>
       <c r="C41" s="13" t="s">
@@ -3097,10 +2501,10 @@
       </c>
       <c r="K41" s="9"/>
     </row>
-    <row r="42" ht="15.75" spans="1:11">
+    <row r="42" spans="1:11" ht="45">
       <c r="A42" s="2"/>
       <c r="B42" s="7">
-        <f>ROW(B42)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>40</v>
       </c>
       <c r="C42" s="13" t="s">
@@ -3127,12 +2531,14 @@
       <c r="J42" s="9">
         <v>1</v>
       </c>
-      <c r="K42" s="9"/>
-    </row>
-    <row r="43" ht="24.75" spans="1:11">
+      <c r="K42" s="15" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="30">
       <c r="A43" s="2"/>
       <c r="B43" s="7">
-        <f>ROW(B43)-ROW($B$2)</f>
+        <f t="shared" si="0"/>
         <v>41</v>
       </c>
       <c r="C43" s="13" t="s">
@@ -3159,14 +2565,19 @@
       <c r="J43" s="9">
         <v>1</v>
       </c>
-      <c r="K43" s="9"/>
+      <c r="K43" s="15" t="s">
+        <v>220</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="I1:K1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="K42" r:id="rId1"/>
+    <hyperlink ref="K43" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>